<commit_message>
Auto commit 17-03-2026 12:19:48.76
</commit_message>
<xml_diff>
--- a/Data Base/Local Templates/gwdtvm/110mm Borewell Construction.xlsx
+++ b/Data Base/Local Templates/gwdtvm/110mm Borewell Construction.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E06EB8-8A98-400A-9530-FFBC9DD9713D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>110mm (4.5") Borewell Drilling (Code: GWDDR100)</t>
   </si>
@@ -27,11 +28,14 @@
   <si>
     <t>PVC End cap 140 mm (DG) (Code: GWDMR003)</t>
   </si>
+  <si>
+    <t>Water Quality Testing (Code: GWDDR462)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -103,6 +107,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -150,7 +157,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -183,9 +190,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -218,6 +242,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -393,15 +434,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="91" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="78" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -409,7 +450,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="403" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -417,7 +458,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="403" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -425,11 +466,19 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="78" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="52" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="65" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>